<commit_message>
Restore NHB meta-analysis method for 24-article update
</commit_message>
<xml_diff>
--- a/data/SourceData_main_model_covariates_20260723_B1Strong.xlsx
+++ b/data/SourceData_main_model_covariates_20260723_B1Strong.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5d33603b0c784fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_model_audit" sheetId="2" r:id="Refa5af0600e94919"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R07cf8e2b848a432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_model_audit" sheetId="2" r:id="R3bf6f26f79a24cc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -35,8 +35,25 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Times New Roman"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -48,8 +65,18 @@
         <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="12">
+  <x:borders count="14">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -133,11 +160,39 @@
         <x:color rgb="FFD9E1F2"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2F3"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="77">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -237,6 +292,90 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -458,77 +597,67 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="96" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="48" t="str">
         <x:v>Main-model covariate audit update - 24 July 2026</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
-        <x:v>Main-model covariate audit update - 24 July 2026</x:v>
-      </x:c>
-      <x:c r="C1" s="4" t="str">
-        <x:v>Main-model covariate audit update - 24 July 2026</x:v>
-      </x:c>
-      <x:c r="D1" s="4" t="str">
-        <x:v>Main-model covariate audit update - 24 July 2026</x:v>
-      </x:c>
-      <x:c r="E1" s="4" t="str">
-        <x:v>Main-model covariate audit update - 24 July 2026</x:v>
-      </x:c>
-      <x:c r="F1" s="4" t="str">
-        <x:v>Main-model covariate audit update - 24 July 2026</x:v>
-      </x:c>
+      <x:c r="B1" s="48"/>
+      <x:c r="C1" s="48"/>
+      <x:c r="D1" s="48"/>
+      <x:c r="E1" s="48"/>
+      <x:c r="F1" s="48"/>
     </x:row>
     <x:row r="2"/>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="10" t="str">
+      <x:c r="A3" s="50" t="str">
         <x:v>Item</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="B3" s="50" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="24" t="str">
+      <x:c r="A4" s="54" t="str">
         <x:v>Rows</x:v>
       </x:c>
-      <x:c r="B4" s="25" t="str">
-        <x:v>39 effect-estimate rows from 24 articles. Liew 2016a ASD is retained as a separate article.</x:v>
+      <x:c r="B4" s="55" t="str">
+        <x:v>39 effect-estimate rows from 24 articles.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
-      <x:c r="A5" s="26" t="str">
+      <x:c r="A5" s="54" t="str">
         <x:v>Scoring</x:v>
       </x:c>
-      <x:c r="B5" s="27" t="str">
+      <x:c r="B5" s="55" t="str">
         <x:v>Only pre-exposure confounder constructs are counted toward B1-B3. Adjusted neonatal/perinatal variables remain documented but are excluded from confounder scoring.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="26" t="str">
-        <x:v>Danish reports</x:v>
-      </x:c>
-      <x:c r="B6" s="27" t="str">
-        <x:v>Liew 2016a ASD and Prahm 2026 are both present. Partial source-population overlap affects dependence modeling, not article inclusion.</x:v>
+      <x:c r="A6" s="54" t="str">
+        <x:v>Prahm</x:v>
+      </x:c>
+      <x:c r="B6" s="55" t="str">
+        <x:v>The exposure-discordant sibling cohort receives B1 Strong under the design-gated rule.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="26" t="str">
-        <x:v>Prahm</x:v>
-      </x:c>
-      <x:c r="B7" s="27" t="str">
-        <x:v>The exposure-discordant sibling cohort receives B1 Strong under the design-gated rule; a B1 Moderate downgrade is reported as sensitivity analysis.</x:v>
+      <x:c r="A7" s="54" t="str">
+        <x:v>Luo</x:v>
+      </x:c>
+      <x:c r="B7" s="55" t="str">
+        <x:v>Family-stratified Cox models receive B1 Strong. Conventional full-cohort Cox models receive B1 Moderate.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="28" t="str">
-        <x:v>Luo</x:v>
-      </x:c>
-      <x:c r="B8" s="29" t="str">
-        <x:v>Family-stratified Cox models receive B1 Strong. Conventional full-cohort Cox models receive B1 Moderate.</x:v>
+      <x:c r="A8" s="54" t="str">
+        <x:v>Search date</x:v>
+      </x:c>
+      <x:c r="B8" s="55" t="str">
+        <x:v>MEDLINE via PubMed and Embase searched from inception through 1 July 2026.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -584,150 +713,150 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="24" t="str">
+      <x:c r="A2" s="65" t="str">
         <x:v>24566677_ADHD</x:v>
       </x:c>
-      <x:c r="B2" s="42" t="str">
+      <x:c r="B2" s="66" t="str">
         <x:v>24566677</x:v>
       </x:c>
-      <x:c r="C2" s="42" t="str">
+      <x:c r="C2" s="66" t="str">
         <x:v>Liew 2014</x:v>
       </x:c>
-      <x:c r="D2" s="42" t="str">
+      <x:c r="D2" s="66" t="str">
         <x:v>ADHD (medication)</x:v>
       </x:c>
-      <x:c r="E2" s="42" t="str">
+      <x:c r="E2" s="66" t="str">
         <x:v>DNBC Cox PH, ADHD medication registry</x:v>
       </x:c>
-      <x:c r="F2" s="42" t="str">
+      <x:c r="F2" s="66" t="str">
         <x:v>SES, adhd, anxiety, apap, birth_weight, birth_year, child_sex, childhood_psychi, depression, drinking, family_problem, fever, ges_age, inflamm_infection, life_crisis, mat_psychi, maternal_age, muscle_joint_dis, other_mental, parent_behavior_score, parity, pre_bmi, smoking</x:v>
       </x:c>
-      <x:c r="G2" s="42" t="str">
+      <x:c r="G2" s="66" t="str">
         <x:v>maternal_age; child_sex; birth_year; gestational_age; birth_weight; parity; SES; smoking; alcohol; prepreg_BMI; maternal_psychiatric_illness; muscle_joint_disease; fever; infection/inflammation</x:v>
       </x:c>
-      <x:c r="H2" s="42" t="str">
+      <x:c r="H2" s="66" t="str">
         <x:v>- parent_behavior_score: used only in SDQ-ADHD-like analysis; not in HKD/medication main model</x:v>
       </x:c>
-      <x:c r="I2" s="25" t="str">
+      <x:c r="I2" s="67" t="str">
         <x:v>Paternal age, Apgar, season of conception evaluated but NOT in final model per text. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="60" hidden="0" customHeight="1">
-      <x:c r="A3" s="26" t="str">
+      <x:c r="A3" s="68" t="str">
         <x:v>26688372_ASD</x:v>
       </x:c>
-      <x:c r="B3" s="43" t="str">
+      <x:c r="B3" s="69" t="str">
         <x:v>26688372</x:v>
       </x:c>
-      <x:c r="C3" s="43" t="str">
+      <x:c r="C3" s="69" t="str">
         <x:v>Liew 2016 (Autism Research)</x:v>
       </x:c>
-      <x:c r="D3" s="43" t="str">
+      <x:c r="D3" s="69" t="str">
         <x:v>ASD</x:v>
       </x:c>
-      <x:c r="E3" s="43" t="str">
+      <x:c r="E3" s="69" t="str">
         <x:v>DNBC Cox PH (fully adjusted)</x:v>
       </x:c>
-      <x:c r="F3" s="43" t="str">
+      <x:c r="F3" s="69" t="str">
         <x:v>NSAIDs, anti_depress, antibiotics, apap, asd, birth_weight, child_birth_year, child_sex, drinking, education, folic_acid, ges_age, infection_inflammation, maternal_age, maternal_bmi, maternal_fever, maternal_psych, muscle/joint_disease, occupation, parity, ses, sleep_meds, smoking</x:v>
       </x:c>
-      <x:c r="G3" s="43" t="str">
+      <x:c r="G3" s="69" t="str">
         <x:v>child_sex; birth_year; maternal_age; parity; SES; smoking; alcohol; prepreg_BMI; folic_acid; maternal_psychiatric_illness; muscle_joint_disease; fever; infection/inflammation; ibuprofen; aspirin</x:v>
       </x:c>
-      <x:c r="H3" s="43" t="str">
+      <x:c r="H3" s="69" t="str">
         <x:v>- anti_depress: sensitivity analysis only
 - antibiotics: sensitivity analysis only
 - sleep_meds: sensitivity analysis only
 - birth_weight: explicitly excluded from final model as potential mediator
 - ges_age: explicitly excluded from final model as potential mediator</x:v>
       </x:c>
-      <x:c r="I3" s="27" t="str">
+      <x:c r="I3" s="70" t="str">
         <x:v>Text: "Birth weight and gestational age are potential mediators... we did not include them in the final model." || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="26" t="str">
+      <x:c r="A4" s="68" t="str">
         <x:v>27353198_ADHD</x:v>
       </x:c>
-      <x:c r="B4" s="43" t="str">
+      <x:c r="B4" s="69" t="str">
         <x:v>27353198</x:v>
       </x:c>
-      <x:c r="C4" s="43" t="str">
+      <x:c r="C4" s="69" t="str">
         <x:v>Avella Garcia 2016</x:v>
       </x:c>
-      <x:c r="D4" s="43" t="str">
+      <x:c r="D4" s="69" t="str">
         <x:v>ADHD (DSM-IV hyp/imp)</x:v>
       </x:c>
-      <x:c r="E4" s="43" t="str">
+      <x:c r="E4" s="69" t="str">
         <x:v>Negative binomial regression for ADHD-DSM-IV hyperactivity/impulsivity</x:v>
       </x:c>
-      <x:c r="F4" s="43" t="str">
+      <x:c r="F4" s="69" t="str">
         <x:v>APAP, ASD/ADHD, IQ, child_age, child_sex, chronic_illness, education, fever, ges_age, other_medication, quality_of_test, region, social_class, urinary_tract_infection</x:v>
       </x:c>
-      <x:c r="G4" s="43" t="str">
+      <x:c r="G4" s="69" t="str">
         <x:v>region/cohort; child_sex; age_at_testing; gestational_age; social_class; maternal_education; maternal_IQ; chronic_illness; fever; urinary_tract_infection; other_medication</x:v>
       </x:c>
-      <x:c r="H4" s="43" t="str">
+      <x:c r="H4" s="69" t="str">
         <x:v>- quality_of_test: Step10 vision verification (2026-04-23): Methods explicitly state quality_of_test is applied ONLY for BSID and MSCA outcomes (1-year cognitive/motor), NOT for 5-year ADHD-DSM-IV hyp/imp (the meta-pooled outcome). Table 2 footnote "b" for ADHD rows confirms: 10 core covariates + use of any other medication = 11; quality_of_test absent.</x:v>
       </x:c>
-      <x:c r="I4" s="27" t="str">
+      <x:c r="I4" s="70" t="str">
         <x:v>Step10 vision verification (2026-04-23, via claude.ai reading of Tables 2/3): Main model for ADHD-DSM-IV hyp/imp (IRR=1.41) has 11 covariates: region(cohort), child_sex(gender), child_age(age_at_testing), ges_age, social_class, education, IQ, chronic_illness, fever, UTI, other_medication. Quality_of_test only applies to BSID/MSCA (1-year) outcomes. K-CPT and CAST rows in Table 2 drop other_medication. Appendix 4 (P&lt;0.20 + 5%-change screen) not in main PDF. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
-      <x:c r="A5" s="26" t="str">
+      <x:c r="A5" s="68" t="str">
         <x:v>27533796_ADHD</x:v>
       </x:c>
-      <x:c r="B5" s="43" t="str">
+      <x:c r="B5" s="69" t="str">
         <x:v>27533796</x:v>
       </x:c>
-      <x:c r="C5" s="43" t="str">
+      <x:c r="C5" s="69" t="str">
         <x:v>Stergiakouli 2016</x:v>
       </x:c>
-      <x:c r="D5" s="43" t="str">
+      <x:c r="D5" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E5" s="43" t="str">
+      <x:c r="E5" s="69" t="str">
         <x:v>ALSPAC; OLS for APAP at 32 weeks</x:v>
       </x:c>
-      <x:c r="F5" s="43" t="str">
+      <x:c r="F5" s="69" t="str">
         <x:v>SES, adhd, apap, apap_partner, apap_post, drinking, genetic_PRS, headache, infection, maternal_age, maternal_psych, migraine, muscle_joint_dis, parity, prepreg_bmi, smoking</x:v>
       </x:c>
-      <x:c r="G5" s="43" t="str">
+      <x:c r="G5" s="69" t="str">
         <x:v>maternal_age; parity; SES; smoking; alcohol; prepreg_BMI; maternal_psychiatric_illness; muscle_joint_disease; infection; migraine; headache</x:v>
       </x:c>
-      <x:c r="H5" s="43" t="str">
+      <x:c r="H5" s="69" t="str">
         <x:v>- apap_partner: negative-control exposure (partner APAP), not a covariate in main model
 - apap_post: negative-control exposure (postnatal APAP), not a covariate in main model
 - genetic_PRS: separate confounding analysis (PRS ~ APAP use); not in main regression</x:v>
       </x:c>
-      <x:c r="I5" s="27" t="str">
+      <x:c r="I5" s="70" t="str">
         <x:v>PRS analysis is a separate test of whether genetic confounding is plausible. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="144" hidden="0" customHeight="1">
-      <x:c r="A6" s="26" t="str">
+      <x:c r="A6" s="68" t="str">
         <x:v>28031314_ADHD</x:v>
       </x:c>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="69" t="str">
         <x:v>28031314</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="69" t="str">
         <x:v>Liew 2016 (IJE, LDPS)</x:v>
       </x:c>
-      <x:c r="D6" s="43" t="str">
+      <x:c r="D6" s="69" t="str">
         <x:v>Attention/executive function (age 5)</x:v>
       </x:c>
-      <x:c r="E6" s="43" t="str">
+      <x:c r="E6" s="69" t="str">
         <x:v>DNBC/LDPS weighted logistic (ever vs never prenatal paracetamol)</x:v>
       </x:c>
-      <x:c r="F6" s="43" t="str">
+      <x:c r="F6" s="69" t="str">
         <x:v>LDPS_participation, alcohol_intake_pregnancy, apap_prenatal, aspirin_use, attention_exec_function_5y, birth_location, child_sex, fever_pregnancy, folic_acid_supplement, home_size, ibuprofen_use, infection_inflammation_pregnancy, maternal_IQ, maternal_SES, maternal_age, maternal_marital_status, maternal_mental_health, missing_baseline_interview, organic_eating, pain_musculoskeletal_disease, parental_education_index, parity, paternal_age, planned_pregnancy, prenatal_antidepressant_use, prepreg_BMI, preterm_birth, sampling_alcohol_category, season_conception, smoking_pregnancy, tester_indicator</x:v>
       </x:c>
-      <x:c r="G6" s="43" t="str">
+      <x:c r="G6" s="69" t="str">
         <x:v>parental_education; maternal_IQ; maternal_mental_health; smoking; alcohol; parity; maternal_age; child_sex; prepreg_BMI; pain/musculoskeletal; fever/infection/inflammation; ibuprofen; aspirin; tester</x:v>
       </x:c>
-      <x:c r="H6" s="43" t="str">
+      <x:c r="H6" s="69" t="str">
         <x:v>- LDPS_participation: IPW weight model for selection (not in outcome regression)
 - birth_location: IPW weight covariate only
 - home_size: IPW weight covariate only
@@ -741,122 +870,122 @@
 - season_conception: IPW weight covariate only
 - tester_indicator: test-administrator quality-control adjustment (measurement level)</x:v>
       </x:c>
-      <x:c r="I6" s="27" t="str">
+      <x:c r="I6" s="70" t="str">
         <x:v>Authors use IPW to correct for LDPS sampling and non-participation. Under strict main-model audit, the IPW weight-model variables are separated out; outcome-regression covariates are the classical confounder set plus indications and co-medications. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="26" t="str">
+      <x:c r="A7" s="68" t="str">
         <x:v>29084830_ADHD</x:v>
       </x:c>
-      <x:c r="B7" s="43" t="str">
+      <x:c r="B7" s="69" t="str">
         <x:v>29084830</x:v>
       </x:c>
-      <x:c r="C7" s="43" t="str">
+      <x:c r="C7" s="69" t="str">
         <x:v>Ystrom 2017</x:v>
       </x:c>
-      <x:c r="D7" s="43" t="str">
+      <x:c r="D7" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E7" s="43" t="str">
+      <x:c r="E7" s="69" t="str">
         <x:v>MoBa Cox PH; duration-stratified</x:v>
       </x:c>
-      <x:c r="F7" s="43" t="str">
+      <x:c r="F7" s="69" t="str">
         <x:v>ADHD, APAP, _week_bmi, anxiety, birth_year, depression, drinking, education, indication_conditions, marital_status, maternal_age, parental_adhd, parity, smoking</x:v>
       </x:c>
-      <x:c r="G7" s="43" t="str">
+      <x:c r="G7" s="69" t="str">
         <x:v>birth_year; parental_adhd; alcohol; smoking; anxiety; depression; maternal_education; marital_status; week17_BMI; maternal_age; parity</x:v>
       </x:c>
-      <x:c r="H7" s="43" t="str">
+      <x:c r="H7" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I7" s="27" t="str">
+      <x:c r="I7" s="70" t="str">
         <x:v>Step9 PDF verification (2026-04-22): Methods/Abstract state "After adjusting for maternal use of acetaminophen before pregnancy, familial risk for ADHD, and indications of acetaminophen use". Prepregnancy APAP is a negative-control covariate adjusted in the main model. Added `apap_before_preg`. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" hidden="0" customHeight="1">
-      <x:c r="A8" s="26" t="str">
+      <x:c r="A8" s="68" t="str">
         <x:v>29970852_ADHD</x:v>
       </x:c>
-      <x:c r="B8" s="43" t="str">
+      <x:c r="B8" s="69" t="str">
         <x:v>29970852</x:v>
       </x:c>
-      <x:c r="C8" s="43" t="str">
+      <x:c r="C8" s="69" t="str">
         <x:v>Ji 2018</x:v>
       </x:c>
-      <x:c r="D8" s="43" t="str">
+      <x:c r="D8" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E8" s="43" t="str">
+      <x:c r="E8" s="69" t="str">
         <x:v>Boston Birth Cohort; multinomial logistic, Model 6 (fully adjusted, abstract-featured)</x:v>
       </x:c>
-      <x:c r="F8" s="43" t="str">
+      <x:c r="F8" s="69" t="str">
         <x:v>adhd_dx, alcohol_pre_or_during_preg, apap_maternal_metabolites, birthweight, breastfeeding, child_sex, delivery_type, early_childhood_lead, intrauterine_infection_inflammation, maternal_age_delivery, maternal_education, maternal_fever_preg, maternal_hdl, maternal_prepreg_bmi, maternal_race_ethnicity, parity, preterm_birth, smoking_pre_or_during_preg</x:v>
       </x:c>
-      <x:c r="G8" s="43" t="str">
+      <x:c r="G8" s="69" t="str">
         <x:v>maternal_age; race/ethnicity; maternal_education; smoking; alcohol; parity; prepreg_BMI; child_sex; delivery_type; gestational_age; birthweight; maternal_fever; intrauterine_infection/inflammation; breastfeeding</x:v>
       </x:c>
-      <x:c r="H8" s="43" t="str">
+      <x:c r="H8" s="69" t="str">
         <x:v>- early_childhood_lead: stratified analysis only
 - maternal_hdl: stratified analysis only
 - preterm_birth: NOT in Ji 2018 adjusted models — they use gestational_age continuous; excluded per Methods §2.5 wording</x:v>
       </x:c>
-      <x:c r="I8" s="27" t="str">
+      <x:c r="I8" s="70" t="str">
         <x:v>Step12 2026-04-24 (user direction): meta-pooled estimate switched from Model 2 (OR=1.91) to Model 6 (OR=1.88) — the "fully adjusted" model featured in the abstract. Model 6 adds maternal_fever, intrauterine_infection/inflammation, and breastfeeding to the Model 2 covariates. Consequence: fever + infection are main-model indication covariates (B2 Weak → Moderate); breastfeeding is a legitimately-adjusted main-model covariate (K_breastfeeding node reinstated with Ji 2018). Stratified analyses (childhood lead, maternal HDL) remain excluded. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="26" t="str">
+      <x:c r="A9" s="68" t="str">
         <x:v>30458756_ADHD</x:v>
       </x:c>
-      <x:c r="B9" s="43" t="str">
+      <x:c r="B9" s="69" t="str">
         <x:v>30458756</x:v>
       </x:c>
-      <x:c r="C9" s="43" t="str">
+      <x:c r="C9" s="69" t="str">
         <x:v>Tovo 2018</x:v>
       </x:c>
-      <x:c r="D9" s="43" t="str">
+      <x:c r="D9" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E9" s="43" t="str">
+      <x:c r="E9" s="69" t="str">
         <x:v>Pelotas cohort; fully adjusted logistic</x:v>
       </x:c>
-      <x:c r="F9" s="43" t="str">
+      <x:c r="F9" s="69" t="str">
         <x:v>adhd, analgesic, anxiety, apap, depression, drinking, infection, mat_age, mat_education, mat_skin_color, nation_economy, parity, pre_preg_bmi, sex, smoking</x:v>
       </x:c>
-      <x:c r="G9" s="43" t="str">
+      <x:c r="G9" s="69" t="str">
         <x:v>maternal_age; parity; national_economic_index; maternal_education; smoking; alcohol; maternal_skin_color; infection; prepreg_BMI; maternal_mood_disorder; other_analgesic</x:v>
       </x:c>
-      <x:c r="H9" s="43" t="str">
+      <x:c r="H9" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I9" s="27" t="str">
+      <x:c r="I9" s="70" t="str">
         <x:v>All DAG nodes map to main model. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="120" hidden="0" customHeight="1">
-      <x:c r="A10" s="26" t="str">
+      <x:c r="A10" s="68" t="str">
         <x:v>30923825_ADHD</x:v>
       </x:c>
-      <x:c r="B10" s="43" t="str">
+      <x:c r="B10" s="69" t="str">
         <x:v>30923825</x:v>
       </x:c>
-      <x:c r="C10" s="43" t="str">
+      <x:c r="C10" s="69" t="str">
         <x:v>Liew 2019 (AJE)</x:v>
       </x:c>
-      <x:c r="D10" s="43" t="str">
+      <x:c r="D10" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E10" s="43" t="str">
+      <x:c r="E10" s="69" t="str">
         <x:v>NHS II; negative control exposure analysis (all-periods mutually adjusted)</x:v>
       </x:c>
-      <x:c r="F10" s="43" t="str">
+      <x:c r="F10" s="69" t="str">
         <x:v>adhd, antiinflamm, apap, apap_postnatal, apap_pre_preg, aspirin, child_birth_order, child_birth_year, child_sex, drinking, ges_diabetes, household income, mat_depression, mat_rheumatoid_arthritis, maternal_age, other_kid_adhd, partner_education, preeclampsia, smoking, social_standing, unmeasured_confounding</x:v>
       </x:c>
-      <x:c r="G10" s="43" t="str">
+      <x:c r="G10" s="69" t="str">
         <x:v>maternal_age; child_birth_year; child_birth_order; gestational_diabetes; preeclampsia; aspirin; other_NSAIDs; apap_pre_pregnancy; apap_postnatal</x:v>
       </x:c>
-      <x:c r="H10" s="43" t="str">
+      <x:c r="H10" s="69" t="str">
         <x:v>- child_sex: sex-stratified analyses only, not a model covariate
 - drinking: sensitivity "social+lifestyle" add-on (subset with ~75% response)
 - smoking: sensitivity "social+lifestyle" add-on (subset with ~75% response)
@@ -868,62 +997,62 @@
 - other_kid_adhd: sensitivity precision analysis (restricted to 1993-1999 births)
 - unmeasured_confounding: meta-variable in DAG, not a study-measured covariate</x:v>
       </x:c>
-      <x:c r="I10" s="27" t="str">
+      <x:c r="I10" s="70" t="str">
         <x:v>apap_postnatal and apap_pre_preg are LEGITIMATE main-model terms here because this IS a negative-control exposure analysis with all three periods mutually adjusted. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="26" t="str">
+      <x:c r="A11" s="68" t="str">
         <x:v>31509360_ADHD</x:v>
       </x:c>
-      <x:c r="B11" s="43" t="str">
+      <x:c r="B11" s="69" t="str">
         <x:v>31509360</x:v>
       </x:c>
-      <x:c r="C11" s="43" t="str">
+      <x:c r="C11" s="69" t="str">
         <x:v>Chen 2019</x:v>
       </x:c>
-      <x:c r="D11" s="43" t="str">
+      <x:c r="D11" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E11" s="43" t="str">
+      <x:c r="E11" s="69" t="str">
         <x:v>Nationwide matched case-control (Taiwan LHID); logistic, Model 2</x:v>
       </x:c>
-      <x:c r="F11" s="43" t="str">
+      <x:c r="F11" s="69" t="str">
         <x:v>adhd, apap, child_age, child_sex, comorbid_perinatal_condition, ges_infection, income, mat_mental, maternal_age, urbanization</x:v>
       </x:c>
-      <x:c r="G11" s="43" t="str">
+      <x:c r="G11" s="69" t="str">
         <x:v>child_age; child_sex; income; urbanization; gestational_infections; comorbid_perinatal_conditions; maternal_mental_health_disorders</x:v>
       </x:c>
-      <x:c r="H11" s="43" t="str">
+      <x:c r="H11" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I11" s="27" t="str">
+      <x:c r="I11" s="70" t="str">
         <x:v>Abstract-level pooled effect (OR 1.20 any trimester) is from Model 2 (fully adjusted, mental-health-inclusive). child_age = matching variable. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="120" hidden="0" customHeight="1">
-      <x:c r="A12" s="26" t="str">
+      <x:c r="A12" s="68" t="str">
         <x:v>31664451_ADHD</x:v>
       </x:c>
-      <x:c r="B12" s="43" t="str">
+      <x:c r="B12" s="69" t="str">
         <x:v>31664451</x:v>
       </x:c>
-      <x:c r="C12" s="43" t="str">
+      <x:c r="C12" s="69" t="str">
         <x:v>Ji 2019</x:v>
       </x:c>
-      <x:c r="D12" s="43" t="str">
+      <x:c r="D12" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E12" s="43" t="str">
+      <x:c r="E12" s="69" t="str">
         <x:v>Boston Birth Cohort; adjusted logistic with cord plasma APAP burden tertiles</x:v>
       </x:c>
-      <x:c r="F12" s="43" t="str">
+      <x:c r="F12" s="69" t="str">
         <x:v>alcohol, apap, asd/adhd, breastfeeding, child_age_last_visit, child_lead, child_sex, cord_apap, delivery_type, education, illicit_drug, inclusion, infection_inflammation, low_bw, marital, mat_adhd, mat_anxiety, mat_depression, maternal_age, maternal_bmi, maternal_fever, parity, preterm_birth, race, smoking, stress</x:v>
       </x:c>
-      <x:c r="G12" s="43" t="str">
+      <x:c r="G12" s="69" t="str">
         <x:v>maternal_age; race/ethnicity; education; marital_status; stress; smoking; alcohol; maternal_bmi; parity; child_sex; delivery_type; preterm_birth; low_birth_weight</x:v>
       </x:c>
-      <x:c r="H12" s="43" t="str">
+      <x:c r="H12" s="69" t="str">
         <x:v>- breastfeeding: stratified analysis only (advisor-flagged)
 - child_age_last_visit: stratified analysis only
 - child_lead: stratified analysis only (advisor-flagged)
@@ -935,33 +1064,33 @@
 - mat_anxiety: sensitivity (further adjustment)
 - mat_depression: sensitivity (further adjustment)</x:v>
       </x:c>
-      <x:c r="I12" s="27" t="str">
+      <x:c r="I12" s="70" t="str">
         <x:v>Ji 2019 final adjusted model per text: maternal age, race/ethnicity, education, marital status, stress, smoking, alcohol, BMI, parity, sex, delivery type, preterm birth, low birth weight. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="120" hidden="0" customHeight="1">
-      <x:c r="A13" s="26" t="str">
+      <x:c r="A13" s="68" t="str">
         <x:v>31664451_ASD</x:v>
       </x:c>
-      <x:c r="B13" s="43" t="str">
+      <x:c r="B13" s="69" t="str">
         <x:v>31664451</x:v>
       </x:c>
-      <x:c r="C13" s="43" t="str">
+      <x:c r="C13" s="69" t="str">
         <x:v>Ji 2019</x:v>
       </x:c>
-      <x:c r="D13" s="43" t="str">
+      <x:c r="D13" s="69" t="str">
         <x:v>ASD</x:v>
       </x:c>
-      <x:c r="E13" s="43" t="str">
+      <x:c r="E13" s="69" t="str">
         <x:v>Boston Birth Cohort; adjusted logistic with cord plasma APAP burden tertiles</x:v>
       </x:c>
-      <x:c r="F13" s="43" t="str">
+      <x:c r="F13" s="69" t="str">
         <x:v>alcohol, apap, asd/adhd, breastfeeding, child_age_last_visit, child_lead, child_sex, cord_apap, delivery_type, education, illicit_drug, inclusion, infection_inflammation, low_bw, marital, mat_adhd, mat_anxiety, mat_depression, maternal_age, maternal_bmi, maternal_fever, parity, preterm_birth, race, smoking, stress</x:v>
       </x:c>
-      <x:c r="G13" s="43" t="str">
+      <x:c r="G13" s="69" t="str">
         <x:v>maternal_age; race/ethnicity; education; marital_status; stress; smoking; alcohol; maternal_bmi; parity; child_sex; delivery_type; preterm_birth; low_birth_weight</x:v>
       </x:c>
-      <x:c r="H13" s="43" t="str">
+      <x:c r="H13" s="69" t="str">
         <x:v>- breastfeeding: stratified analysis only
 - child_age_last_visit: stratified analysis only
 - child_lead: stratified analysis only
@@ -973,151 +1102,151 @@
 - mat_anxiety: sensitivity (further adjustment)
 - mat_depression: sensitivity (further adjustment)</x:v>
       </x:c>
-      <x:c r="I13" s="27" t="str">
+      <x:c r="I13" s="70" t="str">
         <x:v>Same adjusted model is used for the ASD outcome row. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
-      <x:c r="A14" s="26" t="str">
+      <x:c r="A14" s="68" t="str">
         <x:v>32986124_ADHD</x:v>
       </x:c>
-      <x:c r="B14" s="43" t="str">
+      <x:c r="B14" s="69" t="str">
         <x:v>32986124</x:v>
       </x:c>
-      <x:c r="C14" s="43" t="str">
+      <x:c r="C14" s="69" t="str">
         <x:v>Baker 2020</x:v>
       </x:c>
-      <x:c r="D14" s="43" t="str">
+      <x:c r="D14" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E14" s="43" t="str">
+      <x:c r="E14" s="69" t="str">
         <x:v>IPTW-weighted logistic; meconium APAP</x:v>
       </x:c>
-      <x:c r="F14" s="43" t="str">
+      <x:c r="F14" s="69" t="str">
         <x:v>adhd, child_sex, drinking, education, familial_income, maternal_adhd, maternal_age, meconium_apap, prepreg_bmi, resting-state brain connectivity, smoking</x:v>
       </x:c>
-      <x:c r="G14" s="43" t="str">
+      <x:c r="G14" s="69" t="str">
         <x:v>maternal_age; prepreg_BMI; smoking; alcohol; education; familial_income; child_sex</x:v>
       </x:c>
-      <x:c r="H14" s="43" t="str">
+      <x:c r="H14" s="69" t="str">
         <x:v>- maternal_adhd: explicitly excluded from final model (N=155 only); ran as sensitivity only
 - resting-state brain connectivity: mediator / secondary outcome, not a covariate</x:v>
       </x:c>
-      <x:c r="I14" s="27" t="str">
+      <x:c r="I14" s="70" t="str">
         <x:v>Text: "maternal ADHD ... was excluded from the final models because data were only available for 155 individuals". || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
-      <x:c r="A15" s="26" t="str">
+      <x:c r="A15" s="68" t="str">
         <x:v>33230558_ADHD</x:v>
       </x:c>
-      <x:c r="B15" s="43" t="str">
+      <x:c r="B15" s="69" t="str">
         <x:v>33230558</x:v>
       </x:c>
-      <x:c r="C15" s="43" t="str">
+      <x:c r="C15" s="69" t="str">
         <x:v>Inoue 2020</x:v>
       </x:c>
-      <x:c r="D15" s="43" t="str">
+      <x:c r="D15" s="69" t="str">
         <x:v>ADHD-like behaviour</x:v>
       </x:c>
-      <x:c r="E15" s="43" t="str">
+      <x:c r="E15" s="69" t="str">
         <x:v>DNBC log-binomial regression; prenatal exposure adjusted (IPSW-weighted)</x:v>
       </x:c>
-      <x:c r="F15" s="43" t="str">
+      <x:c r="F15" s="69" t="str">
         <x:v>apap_prenatal, behavior_problems_age11, child_birth_year, maternal_age, maternal_alcohol_preg, maternal_fever_preg, maternal_infection_inflammation_preg, maternal_muscle_joint_disease_preg, maternal_prepreg_BMI, maternal_psychiatric_illness, maternal_smoking_preg, maternal_sociooccupational_status, parental_childhood_behavior_score, parity, prenatal_NSAID_use, selection_IPSW</x:v>
       </x:c>
-      <x:c r="G15" s="43" t="str">
+      <x:c r="G15" s="69" t="str">
         <x:v>maternal_age; child_birth_year; parity; socio-occupational_status; prepreg_BMI; smoking; alcohol; maternal_psychiatric_illness; muscle_joint_disease; fever; infection/inflammation; NSAID</x:v>
       </x:c>
-      <x:c r="H15" s="43" t="str">
+      <x:c r="H15" s="69" t="str">
         <x:v>- parental_childhood_behavior_score: sensitivity analysis adjusting for parental childhood behaviour problems
 - selection_IPSW: Step9 correction (2026-04-22): Inoue 2020 DOES use IPSW in main analyses ("Stabilized IPSW ... were incorporated in all regression analyses"). However, IPSW-weight-model variables are not outcome-regression covariates; they are design-based selection adjustments. Excluded from main_model_variables for consistency with Liew 2016 IJE and Smith Webb 2023 treatment.</x:v>
       </x:c>
-      <x:c r="I15" s="27" t="str">
+      <x:c r="I15" s="70" t="str">
         <x:v>Step9 PDF verification (2026-04-22): previous rationale "study does NOT use IPSW" was incorrect — IPSW IS the primary analytic method. Variable list unchanged (14 regression-term covariates); only rationale text updated. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="26" t="str">
+      <x:c r="A16" s="68" t="str">
         <x:v>34679367_ADHD</x:v>
       </x:c>
-      <x:c r="B16" s="43" t="str">
+      <x:c r="B16" s="69" t="str">
         <x:v>34679367</x:v>
       </x:c>
-      <x:c r="C16" s="43" t="str">
+      <x:c r="C16" s="69" t="str">
         <x:v>Anand 2021</x:v>
       </x:c>
-      <x:c r="D16" s="43" t="str">
+      <x:c r="D16" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E16" s="43" t="str">
+      <x:c r="E16" s="69" t="str">
         <x:v>Logistic regression using cord plasma APAP biomarkers</x:v>
       </x:c>
-      <x:c r="F16" s="43" t="str">
+      <x:c r="F16" s="69" t="str">
         <x:v>adhd, child_sex, cord_plasma_apap, delivery_type, drinking, low_birthweight, marital_status, maternal_age, maternal_bmi, maternal_education, maternal_fever, maternal_race, parity, preterm_birth, smoking, stress</x:v>
       </x:c>
-      <x:c r="G16" s="43" t="str">
+      <x:c r="G16" s="69" t="str">
         <x:v>maternal_age; parity; race; education; BMI; stress; fever; smoking; alcohol; marital_status; child_sex; delivery_type; preterm_birth; low_birthweight</x:v>
       </x:c>
-      <x:c r="H16" s="43" t="str">
+      <x:c r="H16" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I16" s="27" t="str">
+      <x:c r="I16" s="70" t="str">
         <x:v>All DAG nodes are in the single adjusted model reported. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="26" t="str">
+      <x:c r="A17" s="68" t="str">
         <x:v>36170224_ADHD</x:v>
       </x:c>
-      <x:c r="B17" s="43" t="str">
+      <x:c r="B17" s="69" t="str">
         <x:v>36170224</x:v>
       </x:c>
-      <x:c r="C17" s="43" t="str">
+      <x:c r="C17" s="69" t="str">
         <x:v>Sznajder 2022</x:v>
       </x:c>
-      <x:c r="D17" s="43" t="str">
+      <x:c r="D17" s="69" t="str">
         <x:v>Attention problems</x:v>
       </x:c>
-      <x:c r="E17" s="43" t="str">
+      <x:c r="E17" s="69" t="str">
         <x:v>Multivariable regression, attention problems outcome</x:v>
       </x:c>
-      <x:c r="F17" s="43" t="str">
+      <x:c r="F17" s="69" t="str">
         <x:v>anxiety/depression, apap, attention_problems, drinking, insurance_coverage, maternal_age, stress, thyroid_condition, trouble_sleeping</x:v>
       </x:c>
-      <x:c r="G17" s="43" t="str">
+      <x:c r="G17" s="69" t="str">
         <x:v>trouble_sleeping; thyroid_condition; maternal_age; insurance_coverage; alcohol; anxiety/depression; stress</x:v>
       </x:c>
-      <x:c r="H17" s="43" t="str">
+      <x:c r="H17" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I17" s="27" t="str">
+      <x:c r="I17" s="70" t="str">
         <x:v>Text explicitly lists all these as covariates for the attention outcome. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="96" hidden="0" customHeight="1">
-      <x:c r="A18" s="26" t="str">
+      <x:c r="A18" s="68" t="str">
         <x:v>36937866_ADHD</x:v>
       </x:c>
-      <x:c r="B18" s="43" t="str">
+      <x:c r="B18" s="69" t="str">
         <x:v>36937866</x:v>
       </x:c>
-      <x:c r="C18" s="43" t="str">
+      <x:c r="C18" s="69" t="str">
         <x:v>Smith Webb 2023</x:v>
       </x:c>
-      <x:c r="D18" s="43" t="str">
+      <x:c r="D18" s="69" t="str">
         <x:v>Behaviour (adolescence)</x:v>
       </x:c>
-      <x:c r="E18" s="43" t="str">
+      <x:c r="E18" s="69" t="str">
         <x:v>Weighted log-binomial regression (SIPW)</x:v>
       </x:c>
-      <x:c r="F18" s="43" t="str">
+      <x:c r="F18" s="69" t="str">
         <x:v>apap, behavior_problems_adolescence, drinking, gravidity, headache, infant_sex, marital_status, maternal_age, maternal_education, maternal_race, pain, parity, paternal_age, planned_pregnancy, smoking, upper_respiratory_infection</x:v>
       </x:c>
-      <x:c r="G18" s="43" t="str">
+      <x:c r="G18" s="69" t="str">
         <x:v>maternal_age; maternal_education; marital_status; alcohol; smoking; parity</x:v>
       </x:c>
-      <x:c r="H18" s="43" t="str">
+      <x:c r="H18" s="69" t="str">
         <x:v>- gravidity: SIPW weight model only (selection adjustment), not main regression covariate
 - headache: SIPW weight model only
 - infant_sex: SIPW weight model only
@@ -1127,656 +1256,656 @@
 - pain: sensitivity column "Indication adjusted" in Table 4
 - upper_respiratory_infection: sensitivity column "Indication adjusted" in Table 4</x:v>
       </x:c>
-      <x:c r="I18" s="27" t="str">
+      <x:c r="I18" s="70" t="str">
         <x:v>Primary regression confounders: maternal age, education, marital status, parity, drinking, smoking. SIPW variables live in the weight model, not the outcome regression — separate row may be warranted. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36" hidden="0" customHeight="1">
-      <x:c r="A19" s="26" t="str">
+      <x:c r="A19" s="68" t="str">
         <x:v>37431475_ADHD_pop</x:v>
       </x:c>
-      <x:c r="B19" s="43" t="str">
+      <x:c r="B19" s="69" t="str">
         <x:v>37431475</x:v>
       </x:c>
-      <x:c r="C19" s="43" t="str">
+      <x:c r="C19" s="69" t="str">
         <x:v>Gustavson 2021</x:v>
       </x:c>
-      <x:c r="D19" s="43" t="str">
+      <x:c r="D19" s="69" t="str">
         <x:v>ADHD (population)</x:v>
       </x:c>
-      <x:c r="E19" s="43" t="str">
+      <x:c r="E19" s="69" t="str">
         <x:v>MoBa Cox PH, propensity-score adjusted (population)</x:v>
       </x:c>
-      <x:c r="F19" s="43" t="str">
+      <x:c r="F19" s="69" t="str">
         <x:v>adhd, apap, apap_after_preg, apap_before_preg, birth_year, child_sex, chronic_autoimmune/inflammatory, depression and anxiety, drinking, familial_confounding, fever/infection, maternal_age, maternal_education, pain, parity, smoking</x:v>
       </x:c>
-      <x:c r="G19" s="43" t="str">
+      <x:c r="G19" s="69" t="str">
         <x:v>indication_groups(pain;fever/infection;chronic_autoimmune/inflammatory;unspecified;other); child_birth_year; maternal_age; alcohol; smoking; anxiety/depression; apap_before&amp;after_pregnancy; n_co-medications; child_sex; maternal_education; parity</x:v>
       </x:c>
-      <x:c r="H19" s="43" t="str">
+      <x:c r="H19" s="69" t="str">
         <x:v>- apap_after_preg: negative-control exposure period, not a covariate
 - apap_before_preg: negative-control exposure period, not a covariate
 - familial_confounding: handled by sibling model, not the population model</x:v>
       </x:c>
-      <x:c r="I19" s="27" t="str">
+      <x:c r="I19" s="70" t="str">
         <x:v>Population model adjusts via propensity score covariates (year, parity, sex, age, education, smoking, alcohol, dep/anx, pain, fever/infection, chronic autoimmune). || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
-      <x:c r="A20" s="26" t="str">
+      <x:c r="A20" s="68" t="str">
         <x:v>37431475_ADHD_sib</x:v>
       </x:c>
-      <x:c r="B20" s="43" t="str">
+      <x:c r="B20" s="69" t="str">
         <x:v>37431475</x:v>
       </x:c>
-      <x:c r="C20" s="43" t="str">
+      <x:c r="C20" s="69" t="str">
         <x:v>Gustavson 2021</x:v>
       </x:c>
-      <x:c r="D20" s="43" t="str">
+      <x:c r="D20" s="69" t="str">
         <x:v>ADHD (sibling)</x:v>
       </x:c>
-      <x:c r="E20" s="43" t="str">
+      <x:c r="E20" s="69" t="str">
         <x:v>Sibling-control model (within-family effect)</x:v>
       </x:c>
-      <x:c r="F20" s="43" t="str">
+      <x:c r="F20" s="69" t="str">
         <x:v>adhd, apap, apap_after_preg, apap_before_preg, birth_year, child_sex, chronic_autoimmune/inflammatory, depression and anxiety, drinking, familial_confounding, fever/infection, maternal_age, maternal_education, pain, parity, smoking</x:v>
       </x:c>
-      <x:c r="G20" s="43" t="str">
+      <x:c r="G20" s="69" t="str">
         <x:v>indication_groups(pain;fever/infection;chronic_autoimmune/inflammatory;unspecified;other); child_birth_year; maternal_age; alcohol; smoking; anxiety/depression; apap_before&amp;after_pregnancy; n_co-medications; child_sex; family_mean_exposure(家庭固定效应)  （注：同胞模型刻意去掉 maternal_education 与 parity）</x:v>
       </x:c>
-      <x:c r="H20" s="43" t="str">
+      <x:c r="H20" s="69" t="str">
         <x:v>- apap_after_preg: negative-control exposure period, not a covariate
 - apap_before_preg: negative-control exposure period, not a covariate</x:v>
       </x:c>
-      <x:c r="I20" s="27" t="str">
+      <x:c r="I20" s="70" t="str">
         <x:v>Sibling (within-family) model — familial_confounding kept as design-based adjustment (family mean exposure + random family intercept). || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="26" t="str">
+      <x:c r="A21" s="68" t="str">
         <x:v>38592388_ADHD_pop</x:v>
       </x:c>
-      <x:c r="B21" s="43" t="str">
+      <x:c r="B21" s="69" t="str">
         <x:v>38592388</x:v>
       </x:c>
-      <x:c r="C21" s="43" t="str">
+      <x:c r="C21" s="69" t="str">
         <x:v>Ahlqvist 2024</x:v>
       </x:c>
-      <x:c r="D21" s="43" t="str">
+      <x:c r="D21" s="69" t="str">
         <x:v>ADHD (population)</x:v>
       </x:c>
-      <x:c r="E21" s="43" t="str">
+      <x:c r="E21" s="69" t="str">
         <x:v>Nationwide cohort Cox PH (primary analysis)</x:v>
       </x:c>
-      <x:c r="F21" s="43" t="str">
+      <x:c r="F21" s="69" t="str">
         <x:v>NSAID, antenatal_visits, antidepression, antimigraine, antiseizure, apap, asd/adhd, aspirin, birth_year, child_sex, chronic_pain, cohabitation, country, education, family, fever, headache, healthcare_visits_pre_preg, household_income, infection, matenal_age, maternal_adhd, maternal_asd, maternal_bmi, maternal_intellectual_dis, maternal_psyc, migraine, opioid, parity, period_delivery, psycholeptic_drug, residence, rheumatoid_arthritis, smoking</x:v>
       </x:c>
-      <x:c r="G21" s="43" t="str">
+      <x:c r="G21" s="69" t="str">
         <x:v>migraine; chronic_pain; infection; fever; rheumatoid_arthritis; headache; birth_year; period_delivery; child_sex; parity; maternal_age; country; residence; cohabitation; maternal_BMI; smoking; maternal_asd; maternal_adhd; maternal_intellectual_dis; maternal_psychiatric; psycholeptic; antidepressant; antiseizure; healthcare_visits_pre_preg; antenatal_visits; education; household_income; aspirin; NSAID; opioid; antimigraine</x:v>
       </x:c>
-      <x:c r="H21" s="43" t="str">
+      <x:c r="H21" s="69" t="str">
         <x:v>- family: family fixed effects only in sibling model</x:v>
       </x:c>
-      <x:c r="I21" s="27" t="str">
+      <x:c r="I21" s="70" t="str">
         <x:v>Text-documented covariate list maps exhaustively to DAG nodes. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="26" t="str">
+      <x:c r="A22" s="68" t="str">
         <x:v>38592388_ADHD_sib</x:v>
       </x:c>
-      <x:c r="B22" s="43" t="str">
+      <x:c r="B22" s="69" t="str">
         <x:v>38592388</x:v>
       </x:c>
-      <x:c r="C22" s="43" t="str">
+      <x:c r="C22" s="69" t="str">
         <x:v>Ahlqvist 2024</x:v>
       </x:c>
-      <x:c r="D22" s="43" t="str">
+      <x:c r="D22" s="69" t="str">
         <x:v>ADHD (sibling)</x:v>
       </x:c>
-      <x:c r="E22" s="43" t="str">
+      <x:c r="E22" s="69" t="str">
         <x:v>Sibling-comparison Cox regression (family fixed effects)</x:v>
       </x:c>
-      <x:c r="F22" s="43" t="str">
+      <x:c r="F22" s="69" t="str">
         <x:v>NSAID, antenatal_visits, antidepression, antimigraine, antiseizure, apap, asd/adhd, aspirin, birth_year, child_sex, chronic_pain, cohabitation, country, education, family, fever, headache, healthcare_visits_pre_preg, household_income, infection, matenal_age, maternal_adhd, maternal_asd, maternal_bmi, maternal_intellectual_dis, maternal_psyc, migraine, opioid, parity, period_delivery, psycholeptic_drug, residence, rheumatoid_arthritis, smoking</x:v>
       </x:c>
-      <x:c r="G22" s="43" t="str">
+      <x:c r="G22" s="69" t="str">
         <x:v>migraine; chronic_pain; infection; fever; rheumatoid_arthritis; headache; birth_year; period_delivery; child_sex; parity; maternal_age; residence; cohabitation; maternal_BMI; smoking; psycholeptic; antidepressant; antiseizure; healthcare_visits_pre_preg; antenatal_visits; education; household_income; aspirin; NSAID; opioid; antimigraine; + family_stratum(家庭固定效应)</x:v>
       </x:c>
-      <x:c r="H22" s="43" t="str">
+      <x:c r="H22" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I22" s="27" t="str">
+      <x:c r="I22" s="70" t="str">
         <x:v>Sibling model uses family fixed effects in addition to the same covariate set. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="26" t="str">
+      <x:c r="A23" s="68" t="str">
         <x:v>38592388_ASD_pop</x:v>
       </x:c>
-      <x:c r="B23" s="43" t="str">
+      <x:c r="B23" s="69" t="str">
         <x:v>38592388</x:v>
       </x:c>
-      <x:c r="C23" s="43" t="str">
+      <x:c r="C23" s="69" t="str">
         <x:v>Ahlqvist 2024</x:v>
       </x:c>
-      <x:c r="D23" s="43" t="str">
+      <x:c r="D23" s="69" t="str">
         <x:v>ASD (population)</x:v>
       </x:c>
-      <x:c r="E23" s="43" t="str">
+      <x:c r="E23" s="69" t="str">
         <x:v>Nationwide cohort Cox PH (primary analysis)</x:v>
       </x:c>
-      <x:c r="F23" s="43" t="str">
+      <x:c r="F23" s="69" t="str">
         <x:v>NSAID, antenatal_visits, antidepression, antimigraine, antiseizure, apap, asd/adhd, aspirin, birth_year, child_sex, chronic_pain, cohabitation, country, education, family, fever, headache, healthcare_visits_pre_preg, household_income, infection, matenal_age, maternal_adhd, maternal_asd, maternal_bmi, maternal_intellectual_dis, maternal_psyc, migraine, opioid, parity, period_delivery, psycholeptic_drug, residence, rheumatoid_arthritis, smoking</x:v>
       </x:c>
-      <x:c r="G23" s="43" t="str">
+      <x:c r="G23" s="69" t="str">
         <x:v>migraine; chronic_pain; infection; fever; rheumatoid_arthritis; headache; birth_year; period_delivery; child_sex; parity; maternal_age; country; residence; cohabitation; maternal_BMI; smoking; maternal_asd; maternal_adhd; maternal_intellectual_dis; maternal_psychiatric; psycholeptic; antidepressant; antiseizure; healthcare_visits_pre_preg; antenatal_visits; education; household_income; aspirin; NSAID; opioid; antimigraine</x:v>
       </x:c>
-      <x:c r="H23" s="43" t="str">
+      <x:c r="H23" s="69" t="str">
         <x:v>- family: family fixed effects only in sibling model</x:v>
       </x:c>
-      <x:c r="I23" s="27" t="str">
+      <x:c r="I23" s="70" t="str">
         <x:v>Same covariate set used for ASD and ADHD outcomes. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="26" t="str">
+      <x:c r="A24" s="68" t="str">
         <x:v>38592388_ASD_sib</x:v>
       </x:c>
-      <x:c r="B24" s="43" t="str">
+      <x:c r="B24" s="69" t="str">
         <x:v>38592388</x:v>
       </x:c>
-      <x:c r="C24" s="43" t="str">
+      <x:c r="C24" s="69" t="str">
         <x:v>Ahlqvist 2024</x:v>
       </x:c>
-      <x:c r="D24" s="43" t="str">
+      <x:c r="D24" s="69" t="str">
         <x:v>ASD (sibling)</x:v>
       </x:c>
-      <x:c r="E24" s="43" t="str">
+      <x:c r="E24" s="69" t="str">
         <x:v>Sibling-comparison Cox regression (family fixed effects)</x:v>
       </x:c>
-      <x:c r="F24" s="43" t="str">
+      <x:c r="F24" s="69" t="str">
         <x:v>NSAID, antenatal_visits, antidepression, antimigraine, antiseizure, apap, asd/adhd, aspirin, birth_year, child_sex, chronic_pain, cohabitation, country, education, family, fever, headache, healthcare_visits_pre_preg, household_income, infection, matenal_age, maternal_adhd, maternal_asd, maternal_bmi, maternal_intellectual_dis, maternal_psyc, migraine, opioid, parity, period_delivery, psycholeptic_drug, residence, rheumatoid_arthritis, smoking</x:v>
       </x:c>
-      <x:c r="G24" s="43" t="str">
+      <x:c r="G24" s="69" t="str">
         <x:v>migraine; chronic_pain; infection; fever; rheumatoid_arthritis; headache; birth_year; period_delivery; child_sex; parity; maternal_age; residence; cohabitation; maternal_BMI; smoking; psycholeptic; antidepressant; antiseizure; healthcare_visits_pre_preg; antenatal_visits; education; household_income; aspirin; NSAID; opioid; antimigraine; + family_stratum(家庭固定效应)</x:v>
       </x:c>
-      <x:c r="H24" s="43" t="str">
+      <x:c r="H24" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I24" s="27" t="str">
+      <x:c r="I24" s="70" t="str">
         <x:v>Sibling-adjusted (family fixed effects). || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="26" t="str">
+      <x:c r="A25" s="68" t="str">
         <x:v>40898607_ADHD_pop</x:v>
       </x:c>
-      <x:c r="B25" s="43" t="str">
+      <x:c r="B25" s="69" t="str">
         <x:v>40898607</x:v>
       </x:c>
-      <x:c r="C25" s="43" t="str">
+      <x:c r="C25" s="69" t="str">
         <x:v>Okubo 2025</x:v>
       </x:c>
-      <x:c r="D25" s="43" t="str">
+      <x:c r="D25" s="69" t="str">
         <x:v>ADHD (population/PSM)</x:v>
       </x:c>
-      <x:c r="E25" s="43" t="str">
+      <x:c r="E25" s="69" t="str">
         <x:v>Primary analysis: 1:1 PSM; Cox PH (cluster-robust)</x:v>
       </x:c>
-      <x:c r="F25" s="43" t="str">
+      <x:c r="F25" s="69" t="str">
         <x:v>Migraine, SLE, adhd_med, analgesics, apap, asd/adhd, asthma, birth_order, birth_year, chronic_pain, dyslipidemia, family, fever, headache, hypertension, infection, mat_mental, maternal_age, migraine_med, rheumatoid_arthritis, weight</x:v>
       </x:c>
-      <x:c r="G25" s="43" t="str">
+      <x:c r="G25" s="69" t="str">
         <x:v>maternal_age; birth_order; birth_year; prepreg_health_checkup; migraine; headache; chronic_pain; infection; fever; asthma; psychiatric_condition; SLE; rheumatoid_arthritis; hypertension; dyslipidemia; acetaminophen(look-back); antimigraine; NSAIDs; aspirin; antipsychotics; antiemetic; corticosteroids; antibiotics; antihistamine; asthma_drugs; antiepileptics; H2_blocker; PPI; antidiabetics; beta_blockers; CCB; lipid_lowering; antithyroid; ADHD_med; migraine_med</x:v>
       </x:c>
-      <x:c r="H25" s="43" t="str">
+      <x:c r="H25" s="69" t="str">
         <x:v>- family: family stratum only in sibling model</x:v>
       </x:c>
-      <x:c r="I25" s="27" t="str">
+      <x:c r="I25" s="70" t="str">
         <x:v>Text gives broad covariate list including diagnostic histories and pre-pregnancy checkup variables. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="26" t="str">
+      <x:c r="A26" s="68" t="str">
         <x:v>40898607_ADHD_sib</x:v>
       </x:c>
-      <x:c r="B26" s="43" t="str">
+      <x:c r="B26" s="69" t="str">
         <x:v>40898607</x:v>
       </x:c>
-      <x:c r="C26" s="43" t="str">
+      <x:c r="C26" s="69" t="str">
         <x:v>Okubo 2025</x:v>
       </x:c>
-      <x:c r="D26" s="43" t="str">
+      <x:c r="D26" s="69" t="str">
         <x:v>ADHD (sibling)</x:v>
       </x:c>
-      <x:c r="E26" s="43" t="str">
+      <x:c r="E26" s="69" t="str">
         <x:v>Sibling-comparison stratified Cox (family strata)</x:v>
       </x:c>
-      <x:c r="F26" s="43" t="str">
+      <x:c r="F26" s="69" t="str">
         <x:v>Migraine, SLE, adhd_med, analgesics, apap, asd/adhd, asthma, birth_order, birth_year, chronic_pain, dyslipidemia, family, fever, headache, hypertension, infection, mat_mental, maternal_age, migraine_med, rheumatoid_arthritis, weight</x:v>
       </x:c>
-      <x:c r="G26" s="43" t="str">
+      <x:c r="G26" s="69" t="str">
         <x:v>family_stratum(以家庭为层的 stratified Cox)；同胞设计用家庭固定效应替代 PS 匹配，吸收同胞共享的诊断/用药混杂（不再单列 PS 协变量）</x:v>
       </x:c>
-      <x:c r="H26" s="43" t="str">
+      <x:c r="H26" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I26" s="27" t="str">
+      <x:c r="I26" s="70" t="str">
         <x:v>family = family identifier for stratification. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="26" t="str">
+      <x:c r="A27" s="68" t="str">
         <x:v>40898607_ASD_pop</x:v>
       </x:c>
-      <x:c r="B27" s="43" t="str">
+      <x:c r="B27" s="69" t="str">
         <x:v>40898607</x:v>
       </x:c>
-      <x:c r="C27" s="43" t="str">
+      <x:c r="C27" s="69" t="str">
         <x:v>Okubo 2025</x:v>
       </x:c>
-      <x:c r="D27" s="43" t="str">
+      <x:c r="D27" s="69" t="str">
         <x:v>ASD (population/PSM)</x:v>
       </x:c>
-      <x:c r="E27" s="43" t="str">
+      <x:c r="E27" s="69" t="str">
         <x:v>Primary analysis: 1:1 PSM; Cox PH</x:v>
       </x:c>
-      <x:c r="F27" s="43" t="str">
+      <x:c r="F27" s="69" t="str">
         <x:v>Migraine, SLE, adhd_med, analgesics, apap, asd/adhd, asthma, birth_order, birth_year, chronic_pain, dyslipidemia, family, fever, headache, hypertension, infection, mat_mental, maternal_age, migraine_med, rheumatoid_arthritis, weight</x:v>
       </x:c>
-      <x:c r="G27" s="43" t="str">
+      <x:c r="G27" s="69" t="str">
         <x:v>maternal_age; birth_order; birth_year; prepreg_health_checkup; migraine; headache; chronic_pain; infection; fever; asthma; psychiatric_condition; SLE; rheumatoid_arthritis; hypertension; dyslipidemia; acetaminophen(look-back); antimigraine; NSAIDs; aspirin; antipsychotics; antiemetic; corticosteroids; antibiotics; antihistamine; asthma_drugs; antiepileptics; H2_blocker; PPI; antidiabetics; beta_blockers; CCB; lipid_lowering; antithyroid; ADHD_med; migraine_med</x:v>
       </x:c>
-      <x:c r="H27" s="43" t="str">
+      <x:c r="H27" s="69" t="str">
         <x:v>- family: family stratum only in sibling model</x:v>
       </x:c>
-      <x:c r="I27" s="27" t="str">
+      <x:c r="I27" s="70" t="str">
         <x:v>|| [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="26" t="str">
+      <x:c r="A28" s="68" t="str">
         <x:v>40898607_ASD_sib</x:v>
       </x:c>
-      <x:c r="B28" s="43" t="str">
+      <x:c r="B28" s="69" t="str">
         <x:v>40898607</x:v>
       </x:c>
-      <x:c r="C28" s="43" t="str">
+      <x:c r="C28" s="69" t="str">
         <x:v>Okubo 2025</x:v>
       </x:c>
-      <x:c r="D28" s="43" t="str">
+      <x:c r="D28" s="69" t="str">
         <x:v>ASD (sibling)</x:v>
       </x:c>
-      <x:c r="E28" s="43" t="str">
+      <x:c r="E28" s="69" t="str">
         <x:v>Sibling-comparison stratified Cox</x:v>
       </x:c>
-      <x:c r="F28" s="43" t="str">
+      <x:c r="F28" s="69" t="str">
         <x:v>Migraine, SLE, adhd_med, analgesics, apap, asd/adhd, asthma, birth_order, birth_year, chronic_pain, dyslipidemia, family, fever, headache, hypertension, infection, mat_mental, maternal_age, migraine_med, rheumatoid_arthritis, weight</x:v>
       </x:c>
-      <x:c r="G28" s="43" t="str">
+      <x:c r="G28" s="69" t="str">
         <x:v>family_stratum(以家庭为层的 stratified Cox)；同胞设计用家庭固定效应替代 PS 匹配，吸收同胞共享的诊断/用药混杂（不再单列 PS 协变量）</x:v>
       </x:c>
-      <x:c r="H28" s="43" t="str">
+      <x:c r="H28" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I28" s="27" t="str">
+      <x:c r="I28" s="70" t="str">
         <x:v>|| [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
-      <x:c r="A29" s="26" t="str">
+      <x:c r="A29" s="68" t="str">
         <x:v>40964537_ADHD</x:v>
       </x:c>
-      <x:c r="B29" s="43" t="str">
+      <x:c r="B29" s="69" t="str">
         <x:v>40964537</x:v>
       </x:c>
-      <x:c r="C29" s="43" t="str">
+      <x:c r="C29" s="69" t="str">
         <x:v>Baker 2025</x:v>
       </x:c>
-      <x:c r="D29" s="43" t="str">
+      <x:c r="D29" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E29" s="43" t="str">
+      <x:c r="E29" s="69" t="str">
         <x:v>Biomarker-based logistic regression</x:v>
       </x:c>
-      <x:c r="F29" s="43" t="str">
+      <x:c r="F29" s="69" t="str">
         <x:v>NSAID, adhd, antibiotic, apap in maternal plasma, birth_weight, child_age, child_sex, delivery_type, drinking, education, ges_age, gravidity, household_income, labor_type, maternal_age, neigh_depri_index, parent_mental, pre_bmi, race, smoking, stress</x:v>
       </x:c>
-      <x:c r="G29" s="43" t="str">
+      <x:c r="G29" s="69" t="str">
         <x:v>maternal_age; education; ethnicity; prepreg_BMI; alcohol; tobacco; stress; gravidity; delivery_method; labor_type; household_income; neighborhood_deprivation_index; child_age_at_visit; family_mental_health_disorders; child_sex; NSAID; antibiotic</x:v>
       </x:c>
-      <x:c r="H29" s="43" t="str">
+      <x:c r="H29" s="69" t="str">
         <x:v>- birth_weight: sensitivity model only (possible mediator)
 - ges_age: sensitivity model only (possible mediator)</x:v>
       </x:c>
-      <x:c r="I29" s="27" t="str">
+      <x:c r="I29" s="70" t="str">
         <x:v>Step9 PDF verification (2026-04-22): Figure 2 conceptual model places `Gravidity` as a PRECISION VARIABLE, and caption states "primary models adjusted for confounders AND precision variables". Previously excluded gravidity based on absence from the main text covariate sentence; Figure 2 confirms it IS in primary model. Added gravidity. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="26" t="str">
+      <x:c r="A30" s="68" t="str">
         <x:v>41238184_ADHD</x:v>
       </x:c>
-      <x:c r="B30" s="43" t="str">
+      <x:c r="B30" s="69" t="str">
         <x:v>41238184</x:v>
       </x:c>
-      <x:c r="C30" s="43" t="str">
+      <x:c r="C30" s="69" t="str">
         <x:v>Pleau 2026</x:v>
       </x:c>
-      <x:c r="D30" s="43" t="str">
+      <x:c r="D30" s="69" t="str">
         <x:v>ADHD</x:v>
       </x:c>
-      <x:c r="E30" s="43" t="str">
+      <x:c r="E30" s="69" t="str">
         <x:v>Quebec cohort; adjusted Cox PH (clustered SE)</x:v>
       </x:c>
-      <x:c r="F30" s="43" t="str">
+      <x:c r="F30" s="69" t="str">
         <x:v>NSAID, adhd, antepartum_hemorrhage, apap, asthma, birth_year, delivery_age, delivery_type, depression/anxiety, drinking, drug_abuse, drug_coverage, emergency_visit, epilepsy, fever, malpresentation_fetus, maternal_adhd, maternal_diabetes, maternal_hypertension, obesity, obstetrician_followup, opioid, pain, premature_contractions, premature_rupture_membrane, residence, smoking</x:v>
       </x:c>
-      <x:c r="G30" s="43" t="str">
+      <x:c r="G30" s="69" t="str">
         <x:v>maternal_age; residence; drug_coverage; apap_first_trimester; NSAID; opioid; n_other_medications; tobacco_abuse; alcohol_abuse; drug_abuse; obesity; maternal_adhd; chronic_hypertension; gestational_hypertension; diabetes; gestational_diabetes; asthma; epilepsy; depression/anxiety; other_mental_health; pain; fever; obstetrician_followup; emergency_visit; antepartum_hemorrhage; premature_contractions; premature_rupture_membrane; malpresentation; delivery_mode; birth_year; small_for_gestational_age</x:v>
       </x:c>
-      <x:c r="H30" s="43" t="str">
+      <x:c r="H30" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I30" s="27" t="str">
+      <x:c r="I30" s="70" t="str">
         <x:v>Text enumerates every DAG node as a covariate. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="26" t="str">
+      <x:c r="A31" s="68" t="str">
         <x:v>41801232_ADHD_pop</x:v>
       </x:c>
-      <x:c r="B31" s="43" t="str">
+      <x:c r="B31" s="69" t="str">
         <x:v>41801232</x:v>
       </x:c>
-      <x:c r="C31" s="43" t="str">
+      <x:c r="C31" s="69" t="str">
         <x:v>Lee 2026</x:v>
       </x:c>
-      <x:c r="D31" s="43" t="str">
+      <x:c r="D31" s="69" t="str">
         <x:v>ADHD (full cohort)</x:v>
       </x:c>
-      <x:c r="E31" s="43" t="str">
+      <x:c r="E31" s="69" t="str">
         <x:v>Full cohort Cox PH, adjusted</x:v>
       </x:c>
-      <x:c r="F31" s="43" t="str">
+      <x:c r="F31" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="G31" s="43" t="str">
+      <x:c r="G31" s="69" t="str">
         <x:v>maternal_age; parity; employment_status; family_income; urbanization; child_birth_year; child_sex; smoking; alcohol; maternal_inflammation/infection; aspirin_or_ibuprofen(合并1项); maternal_psychiatric_disorders</x:v>
       </x:c>
-      <x:c r="H31" s="43" t="str">
+      <x:c r="H31" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I31" s="27" t="str">
+      <x:c r="I31" s="70" t="str">
         <x:v>From figure 2 footnote: "Models were adjusted for maternal age, parity, employment status, family income, urbanization level, smoking, alcohol consumption, child's birth years, sex, maternal psychiatric disorders, maternal inflammation or infection, and use of aspirin or ibuprofen during pregnancy." Node list is newly extracted; dags.xlsx entry needs to be added. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="26" t="str">
+      <x:c r="A32" s="68" t="str">
         <x:v>41801232_ADHD_sib</x:v>
       </x:c>
-      <x:c r="B32" s="43" t="str">
+      <x:c r="B32" s="69" t="str">
         <x:v>41801232</x:v>
       </x:c>
-      <x:c r="C32" s="43" t="str">
+      <x:c r="C32" s="69" t="str">
         <x:v>Lee 2026</x:v>
       </x:c>
-      <x:c r="D32" s="43" t="str">
+      <x:c r="D32" s="69" t="str">
         <x:v>ADHD (sibling)</x:v>
       </x:c>
-      <x:c r="E32" s="43" t="str">
+      <x:c r="E32" s="69" t="str">
         <x:v>Sibling-matched stratified Cox</x:v>
       </x:c>
-      <x:c r="F32" s="43" t="str">
+      <x:c r="F32" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="G32" s="43" t="str">
+      <x:c r="G32" s="69" t="str">
         <x:v>maternal_age; parity; employment_status; family_income; urbanization; child_birth_year; child_sex; smoking; alcohol; maternal_inflammation/infection; aspirin_or_ibuprofen; maternal_psychiatric_disorders; + family_stratum(家庭分层, cluster-robust SE)</x:v>
       </x:c>
-      <x:c r="H32" s="43" t="str">
+      <x:c r="H32" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I32" s="27" t="str">
+      <x:c r="I32" s="70" t="str">
         <x:v>Same covariate set plus family (sibling-pair) matching stratum. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="26" t="str">
+      <x:c r="A33" s="68" t="str">
         <x:v>41801232_ASD_pop</x:v>
       </x:c>
-      <x:c r="B33" s="43" t="str">
+      <x:c r="B33" s="69" t="str">
         <x:v>41801232</x:v>
       </x:c>
-      <x:c r="C33" s="43" t="str">
+      <x:c r="C33" s="69" t="str">
         <x:v>Lee 2026</x:v>
       </x:c>
-      <x:c r="D33" s="43" t="str">
+      <x:c r="D33" s="69" t="str">
         <x:v>ASD (full cohort)</x:v>
       </x:c>
-      <x:c r="E33" s="43" t="str">
+      <x:c r="E33" s="69" t="str">
         <x:v>Full cohort Cox PH, adjusted</x:v>
       </x:c>
-      <x:c r="F33" s="43" t="str">
+      <x:c r="F33" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="G33" s="43" t="str">
+      <x:c r="G33" s="69" t="str">
         <x:v>maternal_age; parity; employment_status; family_income; urbanization; child_birth_year; child_sex; smoking; alcohol; maternal_inflammation/infection; aspirin_or_ibuprofen; maternal_psychiatric_disorders</x:v>
       </x:c>
-      <x:c r="H33" s="43" t="str">
+      <x:c r="H33" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I33" s="27" t="str">
+      <x:c r="I33" s="70" t="str">
         <x:v>Same covariates, ASD outcome. || [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="26" t="str">
+      <x:c r="A34" s="68" t="str">
         <x:v>41801232_ASD_sib</x:v>
       </x:c>
-      <x:c r="B34" s="43" t="str">
+      <x:c r="B34" s="69" t="str">
         <x:v>41801232</x:v>
       </x:c>
-      <x:c r="C34" s="43" t="str">
+      <x:c r="C34" s="69" t="str">
         <x:v>Lee 2026</x:v>
       </x:c>
-      <x:c r="D34" s="43" t="str">
+      <x:c r="D34" s="69" t="str">
         <x:v>ASD (sibling)</x:v>
       </x:c>
-      <x:c r="E34" s="43" t="str">
+      <x:c r="E34" s="69" t="str">
         <x:v>Sibling-matched stratified Cox</x:v>
       </x:c>
-      <x:c r="F34" s="43" t="str">
+      <x:c r="F34" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="G34" s="43" t="str">
+      <x:c r="G34" s="69" t="str">
         <x:v>maternal_age; parity; employment_status; family_income; urbanization; child_birth_year; child_sex; smoking; alcohol; maternal_inflammation/infection; aspirin_or_ibuprofen; maternal_psychiatric_disorders; + family_stratum(家庭分层, cluster-robust SE)</x:v>
       </x:c>
-      <x:c r="H34" s="43" t="str">
+      <x:c r="H34" s="69" t="str">
         <x:v>NA</x:v>
       </x:c>
-      <x:c r="I34" s="27" t="str">
+      <x:c r="I34" s="70" t="str">
         <x:v>|| [2026-06-12 senior adjudication, PDF-verified: main-model covariates re-set; see 对比表 sheet⑦ for rationale]</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
-      <x:c r="A35" s="26" t="str">
+      <x:c r="A35" s="71" t="str">
         <x:v>41973453_ASD_pop</x:v>
       </x:c>
-      <x:c r="B35" s="43" t="str">
+      <x:c r="B35" s="72" t="str">
         <x:v>41973453</x:v>
       </x:c>
-      <x:c r="C35" s="43" t="str">
+      <x:c r="C35" s="72" t="str">
         <x:v>Prahm 2026</x:v>
       </x:c>
-      <x:c r="D35" s="43" t="str">
+      <x:c r="D35" s="72" t="str">
         <x:v>ASD (population)</x:v>
       </x:c>
-      <x:c r="E35" s="43" t="str">
+      <x:c r="E35" s="72" t="str">
         <x:v>Danish nationwide cohort Cox PH</x:v>
       </x:c>
-      <x:c r="F35" s="43" t="str">
+      <x:c r="F35" s="72" t="str">
         <x:v>maternal_age; calendar_time; prepregnancy_BMI; smoking; country_of_birth; education; income; urban_residence; cohabitation; parity; asthma; chronic_pain; diabetes; headache; fever; fibromyalgia; gastric_bypass; infection; migraine; neuropathic_pain; rheumatoid_arthritis; maternal_psychiatric_disease; aspirin; antidepressant; antimigraine; antiseizure; NSAID; psycholeptic; opioid; healthcare_utilisation; paternal_age; paternal_psychiatric_history; maternal_sibling_psychiatric_history; child_sex; season_of_birth</x:v>
       </x:c>
-      <x:c r="G35" s="43" t="str">
+      <x:c r="G35" s="72" t="str">
         <x:v>maternal_age; calendar_time; prepregnancy_BMI; smoking; country_of_birth; education; income; urban_residence; cohabitation; parity; asthma; chronic_pain; diabetes; headache; fever; fibromyalgia; gastric_bypass; infection; migraine; neuropathic_pain; rheumatoid_arthritis; maternal_psychiatric_disease; aspirin; antidepressant; antimigraine; antiseizure; NSAID; psycholeptic; opioid; healthcare_utilisation; paternal_age; paternal_psychiatric_history; maternal_sibling_psychiatric_history; child_sex; season_of_birth</x:v>
       </x:c>
-      <x:c r="H35" s="43" t="str">
+      <x:c r="H35" s="72" t="str">
         <x:v>OTC acetaminophen purchases were unavailable; exposure is prescription dispensing. Perinatal outcomes were not included as confounder constructs.</x:v>
       </x:c>
-      <x:c r="I35" s="27" t="str">
+      <x:c r="I35" s="73" t="str">
         <x:v>Population model. Full covariate list verified from the Figure footnote in the main article.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="26" t="str">
+      <x:c r="A36" s="71" t="str">
         <x:v>41973453_ASD_sib</x:v>
       </x:c>
-      <x:c r="B36" s="43" t="str">
+      <x:c r="B36" s="72" t="str">
         <x:v>41973453</x:v>
       </x:c>
-      <x:c r="C36" s="43" t="str">
+      <x:c r="C36" s="72" t="str">
         <x:v>Prahm 2026</x:v>
       </x:c>
-      <x:c r="D36" s="43" t="str">
+      <x:c r="D36" s="72" t="str">
         <x:v>ASD (sibling cohort)</x:v>
       </x:c>
-      <x:c r="E36" s="43" t="str">
+      <x:c r="E36" s="72" t="str">
         <x:v>Exposure-discordant sibling sample; Cox model with maternal-ID clustering</x:v>
       </x:c>
-      <x:c r="F36" s="43" t="str">
+      <x:c r="F36" s="72" t="str">
         <x:v>maternal_age; calendar_time; prepregnancy_BMI; smoking; country_of_birth; education; income; urban_residence; cohabitation; parity; asthma; chronic_pain; diabetes; headache; fever; fibromyalgia; gastric_bypass; infection; migraine; neuropathic_pain; rheumatoid_arthritis; maternal_psychiatric_disease; aspirin; antidepressant; antimigraine; antiseizure; NSAID; psycholeptic; opioid; healthcare_utilisation; paternal_age; paternal_psychiatric_history; maternal_sibling_psychiatric_history; child_sex; season_of_birth; maternal_ID_cluster</x:v>
       </x:c>
-      <x:c r="G36" s="43" t="str">
+      <x:c r="G36" s="72" t="str">
         <x:v>maternal_age; calendar_time; prepregnancy_BMI; smoking; country_of_birth; education; income; urban_residence; cohabitation; parity; asthma; chronic_pain; diabetes; headache; fever; fibromyalgia; gastric_bypass; infection; migraine; neuropathic_pain; rheumatoid_arthritis; maternal_psychiatric_disease; aspirin; antidepressant; antimigraine; antiseizure; NSAID; psycholeptic; opioid; healthcare_utilisation; paternal_age; paternal_psychiatric_history; maternal_sibling_psychiatric_history; child_sex; season_of_birth; maternal_ID_cluster</x:v>
       </x:c>
-      <x:c r="H36" s="43" t="str">
+      <x:c r="H36" s="72" t="str">
         <x:v>Fibromyalgia was omitted because of model nonconvergence. The exposure-discordant sibling cohort met the design gate for B1 Strong; maternal-ID clustering was not treated as equivalent to family-stratified/fixed-effects Cox.</x:v>
       </x:c>
-      <x:c r="I36" s="27" t="str">
+      <x:c r="I36" s="73" t="str">
         <x:v>B1 is Strong in the primary rating under the design-gated rule. A downgrade to Moderate is reported as a sensitivity analysis because no family stratum or fixed effect was described.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
-      <x:c r="A37" s="26" t="str">
+      <x:c r="A37" s="71" t="str">
         <x:v>42371637_ADHD_pop</x:v>
       </x:c>
-      <x:c r="B37" s="43" t="str">
+      <x:c r="B37" s="72" t="str">
         <x:v>42371637</x:v>
       </x:c>
-      <x:c r="C37" s="43" t="str">
+      <x:c r="C37" s="72" t="str">
         <x:v>Luo 2026</x:v>
       </x:c>
-      <x:c r="D37" s="43" t="str">
+      <x:c r="D37" s="72" t="str">
         <x:v>ADHD (full cohort)</x:v>
       </x:c>
-      <x:c r="E37" s="43" t="str">
+      <x:c r="E37" s="72" t="str">
         <x:v>Hong Kong conventional Cox PH</x:v>
       </x:c>
-      <x:c r="F37" s="43" t="str">
+      <x:c r="F37" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min</x:v>
       </x:c>
-      <x:c r="G37" s="43" t="str">
+      <x:c r="G37" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min</x:v>
       </x:c>
-      <x:c r="H37" s="43" t="str">
+      <x:c r="H37" s="72" t="str">
         <x:v>Birth trauma, preterm birth, birth weight and Apgar scores were adjusted in the reported model but excluded from confounder scoring as post-exposure/perinatal variables. OTC and private prescriptions were unavailable.</x:v>
       </x:c>
-      <x:c r="I37" s="27" t="str">
+      <x:c r="I37" s="73" t="str">
         <x:v>Same main covariate set as ASD.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
-      <x:c r="A38" s="26" t="str">
+      <x:c r="A38" s="71" t="str">
         <x:v>42371637_ADHD_sib</x:v>
       </x:c>
-      <x:c r="B38" s="43" t="str">
+      <x:c r="B38" s="72" t="str">
         <x:v>42371637</x:v>
       </x:c>
-      <x:c r="C38" s="43" t="str">
+      <x:c r="C38" s="72" t="str">
         <x:v>Luo 2026</x:v>
       </x:c>
-      <x:c r="D38" s="43" t="str">
+      <x:c r="D38" s="72" t="str">
         <x:v>ADHD (sibling)</x:v>
       </x:c>
-      <x:c r="E38" s="43" t="str">
+      <x:c r="E38" s="72" t="str">
         <x:v>Sibling-matched Cox PH stratified by family</x:v>
       </x:c>
-      <x:c r="F38" s="43" t="str">
+      <x:c r="F38" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min; family_stratum</x:v>
       </x:c>
-      <x:c r="G38" s="43" t="str">
+      <x:c r="G38" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min; family_stratum</x:v>
       </x:c>
-      <x:c r="H38" s="43" t="str">
+      <x:c r="H38" s="72" t="str">
         <x:v>Birth trauma, preterm birth, birth weight and Apgar scores were adjusted but excluded from confounder scoring. OTC and private prescriptions were unavailable.</x:v>
       </x:c>
-      <x:c r="I38" s="27" t="str">
+      <x:c r="I38" s="73" t="str">
         <x:v>Same main covariate set as ASD; B1 = Strong.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
-      <x:c r="A39" s="26" t="str">
+      <x:c r="A39" s="71" t="str">
         <x:v>42371637_ASD_pop</x:v>
       </x:c>
-      <x:c r="B39" s="43" t="str">
+      <x:c r="B39" s="72" t="str">
         <x:v>42371637</x:v>
       </x:c>
-      <x:c r="C39" s="43" t="str">
+      <x:c r="C39" s="72" t="str">
         <x:v>Luo 2026</x:v>
       </x:c>
-      <x:c r="D39" s="43" t="str">
+      <x:c r="D39" s="72" t="str">
         <x:v>ASD (full cohort)</x:v>
       </x:c>
-      <x:c r="E39" s="43" t="str">
+      <x:c r="E39" s="72" t="str">
         <x:v>Hong Kong conventional Cox PH</x:v>
       </x:c>
-      <x:c r="F39" s="43" t="str">
+      <x:c r="F39" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min</x:v>
       </x:c>
-      <x:c r="G39" s="43" t="str">
+      <x:c r="G39" s="72" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min</x:v>
       </x:c>
-      <x:c r="H39" s="43" t="str">
+      <x:c r="H39" s="72" t="str">
         <x:v>Birth trauma, preterm birth, birth weight and Apgar scores were adjusted in the reported model but excluded from confounder scoring as post-exposure/perinatal variables. OTC and private prescriptions were unavailable.</x:v>
       </x:c>
-      <x:c r="I39" s="27" t="str">
+      <x:c r="I39" s="73" t="str">
         <x:v>The full-cohort Cox model was selected; propensity-score and IPTW models were sensitivity estimators.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
-      <x:c r="A40" s="28" t="str">
+      <x:c r="A40" s="74" t="str">
         <x:v>42371637_ASD_sib</x:v>
       </x:c>
-      <x:c r="B40" s="44" t="str">
+      <x:c r="B40" s="75" t="str">
         <x:v>42371637</x:v>
       </x:c>
-      <x:c r="C40" s="44" t="str">
+      <x:c r="C40" s="75" t="str">
         <x:v>Luo 2026</x:v>
       </x:c>
-      <x:c r="D40" s="44" t="str">
+      <x:c r="D40" s="75" t="str">
         <x:v>ASD (sibling)</x:v>
       </x:c>
-      <x:c r="E40" s="44" t="str">
+      <x:c r="E40" s="75" t="str">
         <x:v>Sibling-matched Cox PH stratified by family</x:v>
       </x:c>
-      <x:c r="F40" s="44" t="str">
+      <x:c r="F40" s="75" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min; family_stratum</x:v>
       </x:c>
-      <x:c r="G40" s="44" t="str">
+      <x:c r="G40" s="75" t="str">
         <x:v>maternal_age; delivery_year; parity; delivery_mode; maternal_ASD; maternal_ADHD; maternal_intellectual_disability; maternal_psychiatric_disorder; infection; fever; chronic_pain; headache; migraine; asthma; rheumatoid_arthritis; dyslipidemia; chronic_kidney_disease; hypertensive_disease; gestational_hypertension; diabetes; gestational_diabetes; aspirin; NSAID; opioid; antidepressant; antimigraine; antiepileptic; lipid_regulating_drug; antihypertensive; glucose_lowering_agent; child_sex; birth_trauma; preterm_birth; birth_weight; Apgar_1min; Apgar_5min; family_stratum</x:v>
       </x:c>
-      <x:c r="H40" s="44" t="str">
+      <x:c r="H40" s="75" t="str">
         <x:v>Birth trauma, preterm birth, birth weight and Apgar scores were adjusted but excluded from confounder scoring. OTC and private prescriptions were unavailable.</x:v>
       </x:c>
-      <x:c r="I40" s="29" t="str">
+      <x:c r="I40" s="76" t="str">
         <x:v>Family-stratified Cox with cluster-robust standard errors; B1 = Strong.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c9bbcc961d4afd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6833f29c96ce4d33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Sync final 39-estimate submission data
</commit_message>
<xml_diff>
--- a/data/SourceData_main_model_covariates_20260723_B1Strong.xlsx
+++ b/data/SourceData_main_model_covariates_20260723_B1Strong.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R07cf8e2b848a432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_model_audit" sheetId="2" r:id="R3bf6f26f79a24cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf704cb29ae0944a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main_model_audit" sheetId="2" r:id="R89ed166cd64549be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1905,7 +1905,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6833f29c96ce4d33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra432602b3b4c40cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>